<commit_message>
Atualizacao IA executiva e alertas inteligentes
</commit_message>
<xml_diff>
--- a/relatorio_estoque_peps_cmv.xlsx
+++ b/relatorio_estoque_peps_cmv.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -773,13 +773,13 @@
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G8" t="n">
-        <v>136.3</v>
+        <v>49.3</v>
       </c>
       <c r="H8" t="n">
-        <v>2.899999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1218,16 +1218,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Croissant Frango Requeijão</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1247,34 +1247,30 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>12.9</v>
       </c>
       <c r="J2" t="n">
-        <v>77.40000000000001</v>
+        <v>387</v>
       </c>
       <c r="K2" t="n">
-        <v>77.40000000000001</v>
+        <v>387</v>
       </c>
       <c r="L2" t="n">
-        <v>17.4</v>
+        <v>87</v>
       </c>
       <c r="M2" t="n">
         <v>2.9</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1330,7 +1326,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1339,12 +1335,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Açaí</t>
+          <t>Croissant Frango Requeijão</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Açaí</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1359,30 +1355,34 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I4" t="n">
-        <v>16.9</v>
+        <v>12.9</v>
       </c>
       <c r="J4" t="n">
-        <v>84.5</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>84.5</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>27.5</v>
+        <v>17.4</v>
       </c>
       <c r="M4" t="n">
-        <v>5.5</v>
+        <v>2.9</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1932231 - EMBREAGEM VISCOSA</t>
+          <t>Açaí</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mercadoria</t>
+          <t>Açaí</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1411,22 +1411,22 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
         <v>16.9</v>
       </c>
       <c r="J5" t="n">
-        <v>33.8</v>
+        <v>84.5</v>
       </c>
       <c r="K5" t="n">
-        <v>33.8</v>
+        <v>84.5</v>
       </c>
       <c r="L5" t="n">
-        <v>5.800000000000004</v>
+        <v>27.5</v>
       </c>
       <c r="M5" t="n">
-        <v>2.9</v>
+        <v>5.5</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1443,12 +1443,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>1932231 - EMBREAGEM VISCOSA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Mercadoria</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1463,22 +1463,22 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>12.9</v>
+        <v>16.9</v>
       </c>
       <c r="J6" t="n">
-        <v>38.7</v>
+        <v>33.8</v>
       </c>
       <c r="K6" t="n">
-        <v>38.7</v>
+        <v>33.8</v>
       </c>
       <c r="L6" t="n">
-        <v>8.699999999999999</v>
+        <v>5.800000000000004</v>
       </c>
       <c r="M6" t="n">
-        <v>2.899999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Croissant Frango Requeijão</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1515,34 +1515,30 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
         <v>12.9</v>
       </c>
       <c r="J7" t="n">
-        <v>12.9</v>
+        <v>38.7</v>
       </c>
       <c r="K7" t="n">
-        <v>12.9</v>
+        <v>38.7</v>
       </c>
       <c r="L7" t="n">
-        <v>2.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>2.9</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
-        </is>
-      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1551,12 +1547,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pastel Natural Frango</t>
+          <t>Croissant Frango Requeijão</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pastel</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1571,34 +1567,34 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>12.9</v>
       </c>
       <c r="J8" t="n">
-        <v>20.64</v>
+        <v>12.9</v>
       </c>
       <c r="K8" t="n">
-        <v>20.64</v>
+        <v>12.9</v>
       </c>
       <c r="L8" t="n">
-        <v>3.04</v>
+        <v>2.9</v>
       </c>
       <c r="M8" t="n">
-        <v>1.9</v>
+        <v>2.9</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Saída automática por foto de cupom. Detectado: sa PROMOCAO GUARANA NATURAL</t>
+          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1607,12 +1603,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Croissant Frango Requeijão</t>
+          <t>Pastel Natural Frango</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Pastel</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1639,22 +1635,22 @@
         <v>20.64</v>
       </c>
       <c r="L9" t="n">
-        <v>4.64</v>
+        <v>3.04</v>
       </c>
       <c r="M9" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Saída automática por foto de cupom. Detectado: 97 PROMO CROIS FRANGO REQUEIJAO</t>
+          <t>Saída automática por foto de cupom. Detectado: sa PROMOCAO GUARANA NATURAL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1663,12 +1659,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pastel Natural Frango</t>
+          <t>Croissant Frango Requeijão</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pastel</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1686,31 +1682,31 @@
         <v>1.6</v>
       </c>
       <c r="I10" t="n">
-        <v>3.9</v>
+        <v>12.9</v>
       </c>
       <c r="J10" t="n">
-        <v>6.24</v>
+        <v>20.64</v>
       </c>
       <c r="K10" t="n">
-        <v>6.24</v>
+        <v>20.64</v>
       </c>
       <c r="L10" t="n">
-        <v>3.04</v>
+        <v>4.64</v>
       </c>
       <c r="M10" t="n">
-        <v>1.9</v>
+        <v>2.9</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Saída automática por foto de cupom. Detectado: sa PROMOCAO GUARANA NATURAL</t>
+          <t>Saída automática por foto de cupom. Detectado: 97 PROMO CROIS FRANGO REQUEIJAO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1719,12 +1715,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Croissant Frango Requeijão</t>
+          <t>Pastel Natural Frango</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Pastel</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1751,22 +1747,22 @@
         <v>6.24</v>
       </c>
       <c r="L11" t="n">
-        <v>4.64</v>
+        <v>3.04</v>
       </c>
       <c r="M11" t="n">
-        <v>2.899999999999999</v>
+        <v>1.9</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Saída automática por foto de cupom. Detectado: 97 PROMO CROIS FRANGO REQUEIJAO</t>
+          <t>Saída automática por foto de cupom. Detectado: sa PROMOCAO GUARANA NATURAL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1775,46 +1771,54 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Açaí</t>
+          <t>Croissant Frango Requeijão</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Açaí</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>50</v>
+        <v>1.6</v>
       </c>
       <c r="I12" t="n">
-        <v>5.5</v>
+        <v>3.9</v>
       </c>
       <c r="J12" t="n">
-        <v>275</v>
+        <v>6.24</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>6.24</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>4.64</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Saída automática por foto de cupom. Detectado: 97 PROMO CROIS FRANGO REQUEIJAO</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1823,12 +1827,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pastel Natural Frango</t>
+          <t>Açaí</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pastel</t>
+          <t>Açaí</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1842,10 +1846,10 @@
         <v>50</v>
       </c>
       <c r="I13" t="n">
-        <v>1.9</v>
+        <v>5.5</v>
       </c>
       <c r="J13" t="n">
-        <v>95</v>
+        <v>275</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1862,7 +1866,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1871,7 +1875,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pastel Queijo</t>
+          <t>Pastel Natural Frango</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1910,7 +1914,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1919,7 +1923,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pastel Carne</t>
+          <t>Pastel Queijo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1958,7 +1962,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1967,12 +1971,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Croissant Ricota</t>
+          <t>Pastel Carne</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Pastel</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1986,10 +1990,10 @@
         <v>50</v>
       </c>
       <c r="I16" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="J16" t="n">
-        <v>145</v>
+        <v>95</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -2006,7 +2010,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -2015,7 +2019,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Ricota</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2054,7 +2058,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -2063,7 +2067,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2102,7 +2106,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -2111,7 +2115,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Croissant Frango Requeijão</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2121,44 +2125,36 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I19" t="n">
-        <v>12.9</v>
+        <v>2.9</v>
       </c>
       <c r="J19" t="n">
-        <v>12.9</v>
+        <v>145</v>
       </c>
       <c r="K19" t="n">
-        <v>12.9</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -2177,40 +2173,44 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="J20" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="L20" t="n">
         <v>2.9</v>
       </c>
-      <c r="J20" t="n">
-        <v>145</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
       <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Saída automática por foto de cupom. Detectado: ,e6 CROLSSANT INT. FRANGO REQUEIJAO</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -2219,12 +2219,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1932231 - EMBREAGEM VISCOSA</t>
+          <t>Croissant Frango Requeijão</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mercadoria</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2262,55 +2262,59 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pastel Queijo</t>
+          <t>1932231 - EMBREAGEM VISCOSA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Pastel</t>
+          <t>Mercadoria</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="I22" t="n">
-        <v>7.9</v>
+        <v>2.9</v>
       </c>
       <c r="J22" t="n">
-        <v>1185</v>
+        <v>145</v>
       </c>
       <c r="K22" t="n">
-        <v>1185</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2319,7 +2323,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pastel Carne</t>
+          <t>Pastel Queijo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2358,7 +2362,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2377,7 +2381,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2386,16 +2390,16 @@
         <v>150</v>
       </c>
       <c r="I24" t="n">
-        <v>1.7</v>
+        <v>7.9</v>
       </c>
       <c r="J24" t="n">
+        <v>1185</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1185</v>
+      </c>
+      <c r="L24" t="n">
         <v>255</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
@@ -2406,7 +2410,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2415,7 +2419,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pastel Queijo</t>
+          <t>Pastel Carne</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2454,7 +2458,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2463,35 +2467,35 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Croissant Ricota</t>
+          <t>Pastel Queijo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Croissant</t>
+          <t>Pastel</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="I26" t="n">
-        <v>8.9</v>
+        <v>1.7</v>
       </c>
       <c r="J26" t="n">
-        <v>445</v>
+        <v>255</v>
       </c>
       <c r="K26" t="n">
-        <v>445</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -2502,7 +2506,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2511,7 +2515,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Ricota</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2527,19 +2531,19 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="I27" t="n">
-        <v>9.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="J27" t="n">
-        <v>1380</v>
+        <v>445</v>
       </c>
       <c r="K27" t="n">
-        <v>1380</v>
+        <v>445</v>
       </c>
       <c r="L27" t="n">
-        <v>285</v>
+        <v>95</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -2550,7 +2554,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2559,7 +2563,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2578,13 +2582,13 @@
         <v>150</v>
       </c>
       <c r="I28" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J28" t="n">
-        <v>1335</v>
+        <v>1380</v>
       </c>
       <c r="K28" t="n">
-        <v>1335</v>
+        <v>1380</v>
       </c>
       <c r="L28" t="n">
         <v>285</v>
@@ -2598,7 +2602,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2607,7 +2611,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2617,7 +2621,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -2626,31 +2630,27 @@
         <v>150</v>
       </c>
       <c r="I29" t="n">
-        <v>1.9</v>
+        <v>8.9</v>
       </c>
       <c r="J29" t="n">
+        <v>1335</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1335</v>
+      </c>
+      <c r="L29" t="n">
         <v>285</v>
       </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
       <c r="M29" t="n">
         <v>0</v>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2702,7 +2702,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Croissant Ricota</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2721,36 +2721,40 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I31" t="n">
-        <v>8.9</v>
+        <v>1.9</v>
       </c>
       <c r="J31" t="n">
-        <v>890</v>
+        <v>285</v>
       </c>
       <c r="K31" t="n">
-        <v>890</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="N31" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2769,40 +2773,36 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="I32" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="J32" t="n">
+        <v>890</v>
+      </c>
+      <c r="K32" t="n">
+        <v>890</v>
+      </c>
+      <c r="L32" t="n">
+        <v>190</v>
+      </c>
+      <c r="M32" t="n">
         <v>1.9</v>
       </c>
-      <c r="J32" t="n">
-        <v>285</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Ricota</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2821,36 +2821,40 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="I33" t="n">
-        <v>7.9</v>
+        <v>1.9</v>
       </c>
       <c r="J33" t="n">
-        <v>197.5</v>
+        <v>285</v>
       </c>
       <c r="K33" t="n">
-        <v>197.5</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>97.5</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2859,7 +2863,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2875,19 +2879,19 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I34" t="n">
         <v>7.9</v>
       </c>
       <c r="J34" t="n">
-        <v>355.5</v>
+        <v>197.5</v>
       </c>
       <c r="K34" t="n">
-        <v>355.5</v>
+        <v>197.5</v>
       </c>
       <c r="L34" t="n">
-        <v>130.5</v>
+        <v>97.5</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
@@ -2898,7 +2902,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2907,7 +2911,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2923,22 +2927,22 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I35" t="n">
         <v>7.9</v>
       </c>
       <c r="J35" t="n">
-        <v>79</v>
+        <v>355.5</v>
       </c>
       <c r="K35" t="n">
-        <v>79</v>
+        <v>355.5</v>
       </c>
       <c r="L35" t="n">
-        <v>39</v>
+        <v>130.5</v>
       </c>
       <c r="M35" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
@@ -2946,7 +2950,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2955,7 +2959,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2983,10 +2987,10 @@
         <v>79</v>
       </c>
       <c r="L36" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M36" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
@@ -2994,7 +2998,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3003,7 +3007,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3031,10 +3035,10 @@
         <v>79</v>
       </c>
       <c r="L37" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="M37" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
@@ -3042,7 +3046,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3051,7 +3055,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Croissant Queijo Presunto</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3067,22 +3071,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="I38" t="n">
-        <v>6.9</v>
+        <v>7.9</v>
       </c>
       <c r="J38" t="n">
-        <v>310.5</v>
+        <v>79</v>
       </c>
       <c r="K38" t="n">
-        <v>310.5</v>
+        <v>79</v>
       </c>
       <c r="L38" t="n">
-        <v>130.5</v>
+        <v>39</v>
       </c>
       <c r="M38" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
@@ -3090,7 +3094,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3109,28 +3113,28 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="I39" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J39" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="K39" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="L39" t="n">
+        <v>130.5</v>
+      </c>
+      <c r="M39" t="n">
         <v>2.9</v>
-      </c>
-      <c r="J39" t="n">
-        <v>290</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
       </c>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
@@ -3138,7 +3142,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3147,7 +3151,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Croissant Carne</t>
+          <t>Croissant Queijo Presunto</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3157,28 +3161,28 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="I40" t="n">
-        <v>7.9</v>
+        <v>2.9</v>
       </c>
       <c r="J40" t="n">
-        <v>434.5</v>
+        <v>290</v>
       </c>
       <c r="K40" t="n">
-        <v>434.5</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>214.5</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
@@ -3186,7 +3190,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3205,28 +3209,28 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="I41" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="J41" t="n">
+        <v>434.5</v>
+      </c>
+      <c r="K41" t="n">
+        <v>434.5</v>
+      </c>
+      <c r="L41" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="M41" t="n">
         <v>3.9</v>
-      </c>
-      <c r="J41" t="n">
-        <v>390</v>
-      </c>
-      <c r="K41" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0</v>
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
@@ -3234,7 +3238,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3243,31 +3247,35 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>F100E - BATERIA 100AMP</t>
+          <t>Croissant Carne</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Mercadoria</t>
+          <t>Croissant</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="J42" t="n">
+        <v>390</v>
+      </c>
       <c r="K42" t="n">
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>510</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
         <v>0</v>
@@ -3278,7 +3286,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3287,7 +3295,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TC1014 - TAMPA TANQUE ROSCA INT VW MODERNO</t>
+          <t>F100E - BATERIA 100AMP</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3303,7 +3311,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -3311,7 +3319,7 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>59.4</v>
+        <v>510</v>
       </c>
       <c r="M43" t="n">
         <v>0</v>
@@ -3322,7 +3330,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3331,7 +3339,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1932231 - EMBREAGEM VISCOSA</t>
+          <t>TC1014 - TAMPA TANQUE ROSCA INT VW MODERNO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3347,7 +3355,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>0.01</v>
+        <v>0.99</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -3355,10 +3363,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>5.5</v>
+        <v>59.4</v>
       </c>
       <c r="M44" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
@@ -3366,7 +3374,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3391,7 +3399,7 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>0.99</v>
+        <v>0.01</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -3399,7 +3407,7 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>544.5</v>
+        <v>5.5</v>
       </c>
       <c r="M45" t="n">
         <v>550</v>
@@ -3410,7 +3418,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3419,7 +3427,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>F100E - BATERIA 100AMP</t>
+          <t>1932231 - EMBREAGEM VISCOSA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3435,7 +3443,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -3443,10 +3451,10 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>510</v>
+        <v>544.5</v>
       </c>
       <c r="M46" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
@@ -3454,7 +3462,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3463,7 +3471,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TC1014 - TAMPA TANQUE ROSCA INT VW MODERNO</t>
+          <t>F100E - BATERIA 100AMP</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3479,7 +3487,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -3487,10 +3495,10 @@
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>0.6</v>
+        <v>510</v>
       </c>
       <c r="M47" t="n">
-        <v>60</v>
+        <v>510</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
@@ -3498,11 +3506,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3517,48 +3525,32 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>1</v>
-      </c>
-      <c r="I48" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M48" t="n">
         <v>60</v>
       </c>
-      <c r="J48" t="n">
-        <v>60</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>MULTIMARCAS PECAS DIESEL LTDA</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>33260509637385000410550020000482621038100650</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>Entrada automática por XML. Código: 1297 | NCM: 87089990 | CFOP: 5405</t>
-        </is>
-      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3567,7 +3559,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1932231 - EMBREAGEM VISCOSA</t>
+          <t>TC1014 - TAMPA TANQUE ROSCA INT VW MODERNO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3586,10 +3578,10 @@
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>550</v>
+        <v>60</v>
       </c>
       <c r="J49" t="n">
-        <v>550</v>
+        <v>60</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -3612,13 +3604,13 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Entrada automática por XML. Código: 8789 | NCM: 84836019 | CFOP: 5405</t>
+          <t>Entrada automática por XML. Código: 1297 | NCM: 87089990 | CFOP: 5405</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3627,7 +3619,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>F100E - BATERIA 100AMP</t>
+          <t>1932231 - EMBREAGEM VISCOSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3643,13 +3635,13 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
       <c r="J50" t="n">
-        <v>1020</v>
+        <v>550</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -3672,22 +3664,22 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Entrada automática por XML. Código: 14541 | NCM: 85071090 | CFOP: 5405</t>
+          <t>Entrada automática por XML. Código: 8789 | NCM: 84836019 | CFOP: 5405</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CROISSANT INT DE MINAS COM CEB SC 2,5 KG</t>
+          <t>F100E - BATERIA 100AMP</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3703,13 +3695,13 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>80</v>
+        <v>510</v>
       </c>
       <c r="J51" t="n">
-        <v>80</v>
+        <v>1020</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -3722,23 +3714,23 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Forno e Sabor - Folhados e Croissants Ltda</t>
+          <t>MULTIMARCAS PECAS DIESEL LTDA</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>33260360593701000103550000000021961178700803</t>
+          <t>33260509637385000410550020000482621038100650</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>XML Código 001338 NCM 19059090 CFOP 5405</t>
+          <t>Entrada automática por XML. Código: 14541 | NCM: 85071090 | CFOP: 5405</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -3747,7 +3739,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CROISSANT DE PIZZA LIGHT SC C 2,5 KG</t>
+          <t>CROISSANT INT DE MINAS COM CEB SC 2,5 KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3766,10 +3758,10 @@
         <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="J52" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -3792,13 +3784,13 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>XML Código 001008 NCM 19059090 CFOP 5405</t>
+          <t>XML Código 001338 NCM 19059090 CFOP 5405</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -3807,7 +3799,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CROISSANT DE FRANGO COM REQUEIJAO SC 2,8 KG</t>
+          <t>CROISSANT DE PIZZA LIGHT SC C 2,5 KG</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3823,13 +3815,13 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>74</v>
       </c>
       <c r="J53" t="n">
-        <v>222</v>
+        <v>74</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -3852,13 +3844,13 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>XML Código 001002 NCM 19059090 CFOP 5405</t>
+          <t>XML Código 001008 NCM 19059090 CFOP 5405</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -3867,7 +3859,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CROISSANT MISTO SC 2,8 KG</t>
+          <t>CROISSANT DE FRANGO COM REQUEIJAO SC 2,8 KG</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3911,6 +3903,66 @@
         </is>
       </c>
       <c r="P54" t="inlineStr">
+        <is>
+          <t>XML Código 001002 NCM 19059090 CFOP 5405</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CROISSANT MISTO SC 2,8 KG</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Mercadoria</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>3</v>
+      </c>
+      <c r="I55" t="n">
+        <v>74</v>
+      </c>
+      <c r="J55" t="n">
+        <v>222</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Forno e Sabor - Folhados e Croissants Ltda</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>33260360593701000103550000000021961178700803</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
         <is>
           <t>XML Código 001001 NCM 19059090 CFOP 5405</t>
         </is>
@@ -4393,13 +4445,13 @@
         <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G11" t="n">
         <v>2.9</v>
       </c>
       <c r="H11" t="n">
-        <v>136.3</v>
+        <v>49.3</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -5043,31 +5095,31 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>253</v>
+        <v>283</v>
       </c>
       <c r="E3" t="n">
-        <v>2163.7</v>
+        <v>2550.7</v>
       </c>
       <c r="F3" t="n">
-        <v>683.7</v>
+        <v>770.7</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>683.7</v>
+        <v>770.7</v>
       </c>
       <c r="I3" t="n">
-        <v>31.59865045986043</v>
+        <v>30.21523503352022</v>
       </c>
       <c r="J3" t="n">
-        <v>31.59865045986043</v>
+        <v>30.21523503352022</v>
       </c>
       <c r="K3" t="n">
-        <v>1480</v>
+        <v>1780</v>
       </c>
       <c r="L3" t="n">
-        <v>68.40134954013956</v>
+        <v>69.78476496647978</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>